<commit_message>
export analysis data fix
- deleted lots of unneeded code
- fixed several inconsitencies like mismatched lt.30 filters
- added sumscore cape export
-
</commit_message>
<xml_diff>
--- a/information/2025-10-28_Item_Information_Adults.xlsx
+++ b/information/2025-10-28_Item_Information_Adults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Wilken_Arbeitsordner\Clinical_Backbone_RU5389\information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC2B93C-F65D-4553-B12F-D7F5D2E4977D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{727233F6-1838-4D9B-98DC-AB56DFBCF2F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3569" uniqueCount="1432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3599" uniqueCount="1432">
   <si>
     <t>Item</t>
   </si>
@@ -4743,7 +4743,10 @@
     <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="10" width="21.28515625" customWidth="1"/>
+    <col min="5" max="6" width="21.28515625" customWidth="1"/>
+    <col min="7" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10394,6 +10397,12 @@
       <c r="B301" t="s">
         <v>1337</v>
       </c>
+      <c r="E301" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F301" t="s">
+        <v>1421</v>
+      </c>
       <c r="K301" t="s">
         <v>1375</v>
       </c>
@@ -10405,6 +10414,12 @@
       <c r="B302" t="s">
         <v>1337</v>
       </c>
+      <c r="E302" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F302" t="s">
+        <v>1421</v>
+      </c>
       <c r="K302" t="s">
         <v>1375</v>
       </c>
@@ -10416,6 +10431,12 @@
       <c r="B303" t="s">
         <v>1337</v>
       </c>
+      <c r="E303" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F303" t="s">
+        <v>1421</v>
+      </c>
       <c r="K303" t="s">
         <v>1375</v>
       </c>
@@ -10432,6 +10453,12 @@
       <c r="B305" t="s">
         <v>1337</v>
       </c>
+      <c r="E305" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F305" t="s">
+        <v>1421</v>
+      </c>
       <c r="K305" t="s">
         <v>1375</v>
       </c>
@@ -10443,6 +10470,12 @@
       <c r="B306" t="s">
         <v>1337</v>
       </c>
+      <c r="E306" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F306" t="s">
+        <v>1421</v>
+      </c>
       <c r="K306" t="s">
         <v>1375</v>
       </c>
@@ -10454,6 +10487,12 @@
       <c r="B307" t="s">
         <v>1337</v>
       </c>
+      <c r="E307" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F307" t="s">
+        <v>1421</v>
+      </c>
       <c r="K307" t="s">
         <v>1375</v>
       </c>
@@ -10465,6 +10504,12 @@
       <c r="B308" t="s">
         <v>1337</v>
       </c>
+      <c r="E308" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F308" t="s">
+        <v>1421</v>
+      </c>
       <c r="K308" t="s">
         <v>1375</v>
       </c>
@@ -10476,6 +10521,12 @@
       <c r="B309" t="s">
         <v>1337</v>
       </c>
+      <c r="E309" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F309" t="s">
+        <v>1421</v>
+      </c>
       <c r="K309" t="s">
         <v>1375</v>
       </c>
@@ -10487,6 +10538,12 @@
       <c r="B310" t="s">
         <v>1337</v>
       </c>
+      <c r="E310" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F310" t="s">
+        <v>1421</v>
+      </c>
       <c r="K310" t="s">
         <v>1375</v>
       </c>
@@ -10498,6 +10555,12 @@
       <c r="B311" t="s">
         <v>1337</v>
       </c>
+      <c r="E311" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F311" t="s">
+        <v>1421</v>
+      </c>
       <c r="K311" t="s">
         <v>1375</v>
       </c>
@@ -10509,6 +10572,12 @@
       <c r="B312" t="s">
         <v>1337</v>
       </c>
+      <c r="E312" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F312" t="s">
+        <v>1421</v>
+      </c>
       <c r="K312" t="s">
         <v>1375</v>
       </c>
@@ -10520,6 +10589,12 @@
       <c r="B313" t="s">
         <v>1337</v>
       </c>
+      <c r="E313" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F313" t="s">
+        <v>1421</v>
+      </c>
       <c r="K313" t="s">
         <v>1375</v>
       </c>
@@ -10531,6 +10606,12 @@
       <c r="B314" t="s">
         <v>1337</v>
       </c>
+      <c r="E314" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F314" t="s">
+        <v>1421</v>
+      </c>
       <c r="K314" t="s">
         <v>1375</v>
       </c>
@@ -10542,6 +10623,12 @@
       <c r="B315" t="s">
         <v>1337</v>
       </c>
+      <c r="E315" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F315" t="s">
+        <v>1421</v>
+      </c>
       <c r="K315" t="s">
         <v>1375</v>
       </c>
@@ -10552,6 +10639,12 @@
       </c>
       <c r="B316" t="s">
         <v>1337</v>
+      </c>
+      <c r="E316" t="s">
+        <v>1408</v>
+      </c>
+      <c r="F316" t="s">
+        <v>1421</v>
       </c>
       <c r="K316" t="s">
         <v>1375</v>

</xml_diff>

<commit_message>
turned efa analysis into pipeline
deleted lots of unneeded files
</commit_message>
<xml_diff>
--- a/information/2025-10-28_Item_Information_Adults.xlsx
+++ b/information/2025-10-28_Item_Information_Adults.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Wilken_Arbeitsordner\Clinical_Backbone_RU5389\information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{727233F6-1838-4D9B-98DC-AB56DFBCF2F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6B2E58B-F9E0-4A9A-B54A-29F3F9121D8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3599" uniqueCount="1432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3594" uniqueCount="1432">
   <si>
     <t>Item</t>
   </si>
@@ -6664,9 +6664,6 @@
       <c r="H89" t="s">
         <v>1427</v>
       </c>
-      <c r="K89" t="s">
-        <v>1375</v>
-      </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
@@ -6817,9 +6814,6 @@
       <c r="H95" t="s">
         <v>1427</v>
       </c>
-      <c r="K95" t="s">
-        <v>1375</v>
-      </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
@@ -6847,7 +6841,7 @@
         <v>1418</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>99</v>
       </c>
@@ -6870,7 +6864,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>100</v>
       </c>
@@ -6896,7 +6890,7 @@
         <v>1352</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>101</v>
       </c>
@@ -6922,7 +6916,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>102</v>
       </c>
@@ -6948,7 +6942,7 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>103</v>
       </c>
@@ -6971,7 +6965,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>104</v>
       </c>
@@ -6997,7 +6991,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>105</v>
       </c>
@@ -7023,7 +7017,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>106</v>
       </c>
@@ -7049,7 +7043,7 @@
         <v>1420</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>107</v>
       </c>
@@ -7071,11 +7065,8 @@
       <c r="H105" t="s">
         <v>1427</v>
       </c>
-      <c r="K105" t="s">
-        <v>1375</v>
-      </c>
-    </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>108</v>
       </c>
@@ -7101,7 +7092,7 @@
         <v>1418</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>109</v>
       </c>
@@ -7124,7 +7115,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>110</v>
       </c>
@@ -7150,7 +7141,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>111</v>
       </c>
@@ -7172,11 +7163,8 @@
       <c r="H109" t="s">
         <v>1427</v>
       </c>
-      <c r="K109" t="s">
-        <v>1375</v>
-      </c>
-    </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="110" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>112</v>
       </c>
@@ -7202,7 +7190,7 @@
         <v>1418</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>113</v>
       </c>
@@ -7225,7 +7213,7 @@
         <v>1428</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>114</v>
       </c>
@@ -7251,7 +7239,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>115</v>
       </c>
@@ -7277,7 +7265,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>116</v>
       </c>
@@ -7299,11 +7287,8 @@
       <c r="H114" t="s">
         <v>1427</v>
       </c>
-      <c r="K114" t="s">
-        <v>1375</v>
-      </c>
-    </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>117</v>
       </c>
@@ -7329,7 +7314,7 @@
         <v>1350</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>118</v>
       </c>
@@ -7352,7 +7337,7 @@
         <v>1422</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>119</v>
       </c>
@@ -7372,7 +7357,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>120</v>
       </c>
@@ -7392,7 +7377,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>121</v>
       </c>
@@ -7412,7 +7397,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>122</v>
       </c>
@@ -7432,7 +7417,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>123</v>
       </c>
@@ -7452,7 +7437,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>124</v>
       </c>
@@ -7472,7 +7457,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>125</v>
       </c>
@@ -7492,7 +7477,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>126</v>
       </c>
@@ -7512,7 +7497,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>127</v>
       </c>
@@ -7532,7 +7517,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>128</v>
       </c>
@@ -7552,7 +7537,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>129</v>
       </c>
@@ -7572,7 +7557,7 @@
         <v>1405</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>130</v>
       </c>

</xml_diff>